<commit_message>
[Modify][MOS_EXCEL_Learn] add new question 111 and edit question 41,50
</commit_message>
<xml_diff>
--- a/Data/Excel_Learn/Excel_file_moi/41.xlsx
+++ b/Data/Excel_Learn/Excel_file_moi/41.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/975f0e77483dfe31/Desktop/Excel 2019/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Pareto\Khach hang\24. mos\MOS\hauwork\Source\Word_Thi\Word_Thi\bin\Debug\Zip\Enc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DEC9559-FD97-4B35-B8DA-D429683098D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD7E463-D45D-4E12-B7BF-C5EA6BEC7AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30" yWindow="-30" windowWidth="20610" windowHeight="9195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="January" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="March" sheetId="3" r:id="rId3"/>
     <sheet name="Summary" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1" fullPrecision="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,6 +30,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="118">
   <si>
     <t>Humongous Insurance</t>
   </si>
@@ -168,7 +170,7 @@
     <t>Policy Types</t>
   </si>
   <si>
-    <t xml:space="preserve">MP: Multi Policy 
+    <t>MP: Multi Policy 
 SP: Single Policy BP: Business Policy</t>
   </si>
   <si>
@@ -259,7 +261,7 @@
     <t>235J98SIE94JFNT76</t>
   </si>
   <si>
-    <t xml:space="preserve">MP: Multi Policy
+    <t>MP: Multi Policy
 SP: Single Policy</t>
   </si>
   <si>
@@ -374,7 +376,7 @@
     <t>LM9AC668916676766</t>
   </si>
   <si>
-    <t xml:space="preserve">MP: Multi Policy
+    <t>MP: Multi Policy
 SP: Single Policy
 BP: Business Policy</t>
   </si>
@@ -401,8 +403,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,13 +478,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.79995117038483843"/>
+        <bgColor theme="6" tint="0.79995117038483843"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.79995117038483843"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -500,10 +501,10 @@
       <left/>
       <right/>
       <top style="thin">
-        <color theme="6" tint="0.399975585192419"/>
+        <color theme="6" tint="0.39994506668294322"/>
       </top>
       <bottom style="thin">
-        <color theme="6" tint="0.399975585192419"/>
+        <color theme="6" tint="0.39994506668294322"/>
       </bottom>
       <diagonal/>
     </border>
@@ -512,7 +513,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color theme="6" tint="0.399975585192419"/>
+        <color theme="6" tint="0.39994506668294322"/>
       </bottom>
       <diagonal/>
     </border>
@@ -520,7 +521,7 @@
       <left/>
       <right/>
       <top style="thin">
-        <color theme="6" tint="0.399975585192419"/>
+        <color theme="6" tint="0.39994506668294322"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -540,61 +541,61 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" applyFill="1" borderId="1" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="2" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" applyNumberFormat="1" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" applyNumberFormat="1" fontId="0" fillId="3" applyFill="1" borderId="1" applyBorder="1" xfId="0"/>
-    <xf numFmtId="16" applyNumberFormat="1" fontId="0" fillId="0" borderId="1" applyBorder="1" xfId="0"/>
-    <xf numFmtId="16" applyNumberFormat="1" fontId="0" fillId="0" borderId="3" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" applyNumberFormat="1" fontId="0" fillId="3" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" applyNumberFormat="1" fontId="0" fillId="0" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" applyNumberFormat="1" fontId="0" fillId="0" borderId="3" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="4" applyFill="1" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="4" applyFill="1" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" applyFont="1" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,7 +648,7 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
@@ -656,6 +657,8 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -757,7 +760,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -766,8 +769,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -786,7 +787,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -795,8 +796,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -885,7 +884,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -894,8 +893,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -914,7 +911,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -923,8 +920,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -943,7 +938,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -952,8 +947,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -972,7 +965,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -981,8 +974,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1001,7 +992,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -1010,8 +1001,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1030,7 +1019,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -1039,8 +1028,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1059,7 +1046,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
@@ -1068,8 +1055,6 @@
         <bottom style="thin">
           <color theme="6" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1213,7 +1198,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="vi-VN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1279,7 +1264,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr lang="vi-VN"/>
+                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="inEnd"/>
@@ -1405,7 +1390,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="vi-VN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="205819640"/>
@@ -1513,7 +1498,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="vi-VN"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2136,55 +2121,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>849629</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>798830</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>107949</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6B46D19-3840-474C-AAC9-8D35FC1973FC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2418079" y="5066030"/>
-          <a:ext cx="3843549" cy="4097020"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -2228,12 +2164,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A4:G20" totalsRowShown="0">
   <autoFilter ref="A4:G20" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Client ID" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Client ID" dataDxfId="28"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Policy Number "/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="VIN Number"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Renewal Date" dataDxfId="27"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Years as Member" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Policy Type " dataDxfId="24">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Policy Type " dataDxfId="25">
       <calculatedColumnFormula>LEFT(Table1[[#This Row],[Policy Number ]],2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Discount" dataDxfId="24">
@@ -2245,16 +2181,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table3" displayName="Table3" ref="A4:G18" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table3" displayName="Table3" ref="A4:G18" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="A4:G18" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Client ID" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Policy Number " dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="VIN Number" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Renewal Date" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Years as Member" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Policy Type " dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Discount" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Client ID" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Policy Number " dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="VIN Number" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Renewal Date" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Years as Member" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Policy Type " dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Discount" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2264,12 +2200,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table35" displayName="Table35" ref="A4:G24" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
   <autoFilter ref="A4:G24" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Client ID" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Policy Number " dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Client ID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Policy Number " dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="VIN Number" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Renewal Date" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Renewal Date" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Years as Member" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Policy Type " dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Policy Type " dataDxfId="1">
       <calculatedColumnFormula>LEFT(Table35[[#This Row],[Policy Number ]],2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Discount" dataDxfId="0">
@@ -2557,28 +2493,28 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="1" width="11.28515625" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" customWidth="1"/>
-    <col min="3" max="3" bestFit="1" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.9" customHeight="1" s="24" customFormat="1">
+    <row r="1" spans="1:7" s="24" customFormat="1" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -2586,37 +2522,37 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>53303</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="13">
@@ -2634,14 +2570,14 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>23552</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="13">
@@ -2659,11 +2595,11 @@
         <v>No</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>55223</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -2684,14 +2620,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>35220</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="13">
@@ -2709,14 +2645,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>92527</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>19</v>
       </c>
       <c r="D9" s="13">
@@ -2734,14 +2670,14 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
         <v>23253</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="13">
@@ -2759,14 +2695,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="12">
         <v>35225</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="13">
@@ -2784,14 +2720,14 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="12">
         <v>55253</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>25</v>
       </c>
       <c r="D12" s="13">
@@ -2809,14 +2745,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="12">
         <v>41412</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>27</v>
       </c>
       <c r="D13" s="13">
@@ -2834,14 +2770,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
         <v>45896</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="13">
@@ -2859,14 +2795,14 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="12">
         <v>14422</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" t="s">
         <v>31</v>
       </c>
       <c r="D15" s="13">
@@ -2884,14 +2820,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <v>41221</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>33</v>
       </c>
       <c r="D16" s="13">
@@ -2909,14 +2845,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <v>66262</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" t="s">
         <v>35</v>
       </c>
       <c r="D17" s="13">
@@ -2934,14 +2870,14 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="12">
         <v>36362</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" t="s">
         <v>37</v>
       </c>
       <c r="D18" s="13">
@@ -2959,14 +2895,14 @@
         <v>No</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="12">
         <v>63302</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" t="s">
         <v>39</v>
       </c>
       <c r="D19" s="13">
@@ -2984,14 +2920,14 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="12">
         <v>93322</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" t="s">
         <v>41</v>
       </c>
       <c r="D20" s="13">
@@ -3009,7 +2945,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="23" ht="90">
+    <row r="23" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>42</v>
       </c>
@@ -3018,16 +2954,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="2">
     <mergeCell ref="A1:XFD1"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
-  <headerFooter/>
-  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3046,19 +2980,19 @@
     <col min="7" max="7" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.9" customHeight="1" s="24" customFormat="1">
+    <row r="1" spans="1:7" s="24" customFormat="1" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>44</v>
       </c>
@@ -3066,7 +3000,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>3</v>
       </c>
@@ -3089,11 +3023,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>13622</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>45</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -3102,17 +3036,17 @@
       <c r="D5" s="16">
         <v>44614</v>
       </c>
-      <c r="E5" s="0">
+      <c r="E5">
         <v>8</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>15822</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>47</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -3121,17 +3055,17 @@
       <c r="D6" s="17">
         <v>44595</v>
       </c>
-      <c r="E6" s="0">
+      <c r="E6">
         <v>2</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>16308</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>49</v>
       </c>
       <c r="C7" s="14" t="s">
@@ -3140,17 +3074,17 @@
       <c r="D7" s="16">
         <v>44601</v>
       </c>
-      <c r="E7" s="0">
+      <c r="E7">
         <v>12</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>19272</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>51</v>
       </c>
       <c r="C8" s="15" t="s">
@@ -3159,17 +3093,17 @@
       <c r="D8" s="17">
         <v>44601</v>
       </c>
-      <c r="E8" s="0">
+      <c r="E8">
         <v>6</v>
       </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>34521</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>53</v>
       </c>
       <c r="C9" s="4" t="s">
@@ -3178,17 +3112,17 @@
       <c r="D9" s="16">
         <v>44607</v>
       </c>
-      <c r="E9" s="0">
+      <c r="E9">
         <v>2</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>43909</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>55</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -3197,17 +3131,17 @@
       <c r="D10" s="17">
         <v>44612</v>
       </c>
-      <c r="E10" s="0">
+      <c r="E10">
         <v>9</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>61220</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="4" t="s">
@@ -3216,17 +3150,17 @@
       <c r="D11" s="16">
         <v>44606</v>
       </c>
-      <c r="E11" s="0">
+      <c r="E11">
         <v>5</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>61789</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>59</v>
       </c>
       <c r="C12" s="5" t="s">
@@ -3235,17 +3169,17 @@
       <c r="D12" s="17">
         <v>44606</v>
       </c>
-      <c r="E12" s="0">
+      <c r="E12">
         <v>3</v>
       </c>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>77272</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>61</v>
       </c>
       <c r="C13" s="4" t="s">
@@ -3254,17 +3188,17 @@
       <c r="D13" s="16">
         <v>44612</v>
       </c>
-      <c r="E13" s="0">
+      <c r="E13">
         <v>10</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>86448</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" t="s">
         <v>63</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -3273,17 +3207,17 @@
       <c r="D14" s="17">
         <v>44596</v>
       </c>
-      <c r="E14" s="0">
+      <c r="E14">
         <v>2</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>89216</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" t="s">
         <v>65</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -3292,17 +3226,17 @@
       <c r="D15" s="16">
         <v>44620</v>
       </c>
-      <c r="E15" s="0">
+      <c r="E15">
         <v>2</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>90918</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" t="s">
         <v>67</v>
       </c>
       <c r="C16" s="5" t="s">
@@ -3311,17 +3245,17 @@
       <c r="D16" s="17">
         <v>44601</v>
       </c>
-      <c r="E16" s="0">
+      <c r="E16">
         <v>10</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>91319</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" t="s">
         <v>69</v>
       </c>
       <c r="C17" s="4" t="s">
@@ -3330,17 +3264,17 @@
       <c r="D17" s="16">
         <v>44612</v>
       </c>
-      <c r="E17" s="0">
+      <c r="E17">
         <v>3</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="10">
         <v>98308</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" t="s">
         <v>71</v>
       </c>
       <c r="C18" s="10" t="s">
@@ -3349,13 +3283,13 @@
       <c r="D18" s="18">
         <v>44617</v>
       </c>
-      <c r="E18" s="0">
+      <c r="E18">
         <v>5</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
     </row>
-    <row r="21" ht="30">
+    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>42</v>
       </c>
@@ -3364,13 +3298,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="2">
     <mergeCell ref="A1:XFD1"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -3382,28 +3315,28 @@
   <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" bestFit="1" width="16.42578125" customWidth="1"/>
-    <col min="3" max="3" bestFit="1" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" bestFit="1" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" bestFit="1" width="18.28515625" customWidth="1"/>
-    <col min="6" max="6" bestFit="1" width="13.7109375" customWidth="1"/>
-    <col min="7" max="7" bestFit="1" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.9" customHeight="1" s="26" customFormat="1">
+    <row r="1" spans="1:7" s="26" customFormat="1" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" s="12" customFormat="1">
+    <row r="2" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
     </row>
-    <row r="3" s="12" customFormat="1">
+    <row r="3" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>74</v>
       </c>
@@ -3411,7 +3344,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>3</v>
       </c>
@@ -3434,7 +3367,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>98909</v>
       </c>
@@ -3459,7 +3392,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>66770</v>
       </c>
@@ -3484,7 +3417,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>66220</v>
       </c>
@@ -3509,7 +3442,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>96565</v>
       </c>
@@ -3534,7 +3467,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>68679</v>
       </c>
@@ -3559,7 +3492,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>89766</v>
       </c>
@@ -3584,7 +3517,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>66220</v>
       </c>
@@ -3609,7 +3542,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>96565</v>
       </c>
@@ -3634,7 +3567,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>75177</v>
       </c>
@@ -3659,7 +3592,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>68677</v>
       </c>
@@ -3684,7 +3617,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>66808</v>
       </c>
@@ -3709,7 +3642,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>66505</v>
       </c>
@@ -3734,7 +3667,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>22222</v>
       </c>
@@ -3759,7 +3692,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="10">
         <v>76377</v>
       </c>
@@ -3784,7 +3717,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>62829</v>
       </c>
@@ -3809,7 +3742,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>67879</v>
       </c>
@@ -3834,7 +3767,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>77777</v>
       </c>
@@ -3859,7 +3792,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>68998</v>
       </c>
@@ -3884,7 +3817,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>87798</v>
       </c>
@@ -3909,7 +3842,7 @@
         <v>No</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="10">
         <v>89176</v>
       </c>
@@ -3934,7 +3867,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="27" ht="60">
+    <row r="27" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>42</v>
       </c>
@@ -3943,15 +3876,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="2">
     <mergeCell ref="A1:XFD1"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
-  <headerFooter/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3964,64 +3896,58 @@
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" s="28" customFormat="1">
+    <row r="1" spans="1:2" s="28" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>112</v>
       </c>
       <c r="B2" s="25"/>
     </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="0">
+      <c r="B4">
         <v>16</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="0" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="0">
+      <c r="B5">
         <v>14</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>117</v>
       </c>
-      <c r="B6" s="0">
+      <c r="B6">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="2">
     <mergeCell ref="A1:XFD1"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <drawing r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to Alo1234 under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
-For more information about EPPlus, see https://epplussoftware.com/
-
 </file>
</xml_diff>